<commit_message>
modified:   excel_data/Innovation_Fund_Projects_data - 290326.xlsx 	modified:   public/data/meta.json 	modified:   public/data/projects.json
</commit_message>
<xml_diff>
--- a/excel_data/Innovation_Fund_Projects_data - 290326.xlsx
+++ b/excel_data/Innovation_Fund_Projects_data - 290326.xlsx
@@ -4370,36 +4370,27 @@
     <xf numFmtId="0" fontId="20" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -4421,6 +4412,15 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4742,40 +4742,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="75" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="70"/>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="72"/>
+      <c r="H1" s="72"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="72"/>
+      <c r="G2" s="72"/>
+      <c r="H2" s="72"/>
     </row>
     <row r="4" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="69" t="s">
+      <c r="A4" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="70"/>
-      <c r="C4" s="70"/>
-      <c r="D4" s="70"/>
-      <c r="E4" s="70"/>
-      <c r="F4" s="70"/>
-      <c r="G4" s="70"/>
-      <c r="H4" s="70"/>
+      <c r="B4" s="72"/>
+      <c r="C4" s="72"/>
+      <c r="D4" s="72"/>
+      <c r="E4" s="72"/>
+      <c r="F4" s="72"/>
+      <c r="G4" s="72"/>
+      <c r="H4" s="72"/>
     </row>
     <row r="5" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -4792,12 +4792,12 @@
       <c r="B6" s="3">
         <v>62</v>
       </c>
-      <c r="C6" s="70"/>
-      <c r="D6" s="70"/>
-      <c r="E6" s="70"/>
-      <c r="F6" s="70"/>
-      <c r="G6" s="70"/>
-      <c r="H6" s="70"/>
+      <c r="C6" s="72"/>
+      <c r="D6" s="72"/>
+      <c r="E6" s="72"/>
+      <c r="F6" s="72"/>
+      <c r="G6" s="72"/>
+      <c r="H6" s="72"/>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
@@ -4806,12 +4806,12 @@
       <c r="B7" s="5">
         <v>16</v>
       </c>
-      <c r="C7" s="70"/>
-      <c r="D7" s="70"/>
-      <c r="E7" s="70"/>
-      <c r="F7" s="70"/>
-      <c r="G7" s="70"/>
-      <c r="H7" s="70"/>
+      <c r="C7" s="72"/>
+      <c r="D7" s="72"/>
+      <c r="E7" s="72"/>
+      <c r="F7" s="72"/>
+      <c r="G7" s="72"/>
+      <c r="H7" s="72"/>
     </row>
     <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
@@ -4820,12 +4820,12 @@
       <c r="B8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="70"/>
-      <c r="D8" s="70"/>
-      <c r="E8" s="70"/>
-      <c r="F8" s="70"/>
-      <c r="G8" s="70"/>
-      <c r="H8" s="70"/>
+      <c r="C8" s="72"/>
+      <c r="D8" s="72"/>
+      <c r="E8" s="72"/>
+      <c r="F8" s="72"/>
+      <c r="G8" s="72"/>
+      <c r="H8" s="72"/>
     </row>
     <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
@@ -4834,12 +4834,12 @@
       <c r="B9" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="70"/>
-      <c r="D9" s="70"/>
-      <c r="E9" s="70"/>
-      <c r="F9" s="70"/>
-      <c r="G9" s="70"/>
-      <c r="H9" s="70"/>
+      <c r="C9" s="72"/>
+      <c r="D9" s="72"/>
+      <c r="E9" s="72"/>
+      <c r="F9" s="72"/>
+      <c r="G9" s="72"/>
+      <c r="H9" s="72"/>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -4848,12 +4848,12 @@
       <c r="B10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="70"/>
-      <c r="D10" s="70"/>
-      <c r="E10" s="70"/>
-      <c r="F10" s="70"/>
-      <c r="G10" s="70"/>
-      <c r="H10" s="70"/>
+      <c r="C10" s="72"/>
+      <c r="D10" s="72"/>
+      <c r="E10" s="72"/>
+      <c r="F10" s="72"/>
+      <c r="G10" s="72"/>
+      <c r="H10" s="72"/>
     </row>
     <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
@@ -4862,12 +4862,12 @@
       <c r="B11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="70"/>
-      <c r="D11" s="70"/>
-      <c r="E11" s="70"/>
-      <c r="F11" s="70"/>
-      <c r="G11" s="70"/>
-      <c r="H11" s="70"/>
+      <c r="C11" s="72"/>
+      <c r="D11" s="72"/>
+      <c r="E11" s="72"/>
+      <c r="F11" s="72"/>
+      <c r="G11" s="72"/>
+      <c r="H11" s="72"/>
     </row>
     <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
@@ -4876,24 +4876,24 @@
       <c r="B12" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="70"/>
-      <c r="D12" s="70"/>
-      <c r="E12" s="70"/>
-      <c r="F12" s="70"/>
-      <c r="G12" s="70"/>
-      <c r="H12" s="70"/>
+      <c r="C12" s="72"/>
+      <c r="D12" s="72"/>
+      <c r="E12" s="72"/>
+      <c r="F12" s="72"/>
+      <c r="G12" s="72"/>
+      <c r="H12" s="72"/>
     </row>
     <row r="15" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="69" t="s">
+      <c r="A15" s="74" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="70"/>
-      <c r="C15" s="70"/>
-      <c r="D15" s="70"/>
-      <c r="E15" s="70"/>
-      <c r="F15" s="70"/>
-      <c r="G15" s="70"/>
-      <c r="H15" s="70"/>
+      <c r="B15" s="72"/>
+      <c r="C15" s="72"/>
+      <c r="D15" s="72"/>
+      <c r="E15" s="72"/>
+      <c r="F15" s="72"/>
+      <c r="G15" s="72"/>
+      <c r="H15" s="72"/>
     </row>
     <row r="16" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -4905,11 +4905,11 @@
       <c r="C16" s="76" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="72"/>
-      <c r="E16" s="72"/>
-      <c r="F16" s="72"/>
-      <c r="G16" s="72"/>
-      <c r="H16" s="73"/>
+      <c r="D16" s="70"/>
+      <c r="E16" s="70"/>
+      <c r="F16" s="70"/>
+      <c r="G16" s="70"/>
+      <c r="H16" s="71"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
@@ -4918,14 +4918,14 @@
       <c r="B17" s="9">
         <v>21</v>
       </c>
-      <c r="C17" s="71" t="s">
+      <c r="C17" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="72"/>
-      <c r="E17" s="72"/>
-      <c r="F17" s="72"/>
-      <c r="G17" s="72"/>
-      <c r="H17" s="73"/>
+      <c r="D17" s="70"/>
+      <c r="E17" s="70"/>
+      <c r="F17" s="70"/>
+      <c r="G17" s="70"/>
+      <c r="H17" s="71"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
@@ -4934,14 +4934,14 @@
       <c r="B18" s="11">
         <v>20</v>
       </c>
-      <c r="C18" s="75" t="s">
+      <c r="C18" s="73" t="s">
         <v>24</v>
       </c>
-      <c r="D18" s="72"/>
-      <c r="E18" s="72"/>
-      <c r="F18" s="72"/>
-      <c r="G18" s="72"/>
-      <c r="H18" s="73"/>
+      <c r="D18" s="70"/>
+      <c r="E18" s="70"/>
+      <c r="F18" s="70"/>
+      <c r="G18" s="70"/>
+      <c r="H18" s="71"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
@@ -4950,14 +4950,14 @@
       <c r="B19" s="13">
         <v>10</v>
       </c>
-      <c r="C19" s="71" t="s">
+      <c r="C19" s="69" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="72"/>
-      <c r="E19" s="72"/>
-      <c r="F19" s="72"/>
-      <c r="G19" s="72"/>
-      <c r="H19" s="73"/>
+      <c r="D19" s="70"/>
+      <c r="E19" s="70"/>
+      <c r="F19" s="70"/>
+      <c r="G19" s="70"/>
+      <c r="H19" s="71"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
@@ -4966,14 +4966,14 @@
       <c r="B20" s="15">
         <v>4</v>
       </c>
-      <c r="C20" s="75" t="s">
+      <c r="C20" s="73" t="s">
         <v>28</v>
       </c>
-      <c r="D20" s="72"/>
-      <c r="E20" s="72"/>
-      <c r="F20" s="72"/>
-      <c r="G20" s="72"/>
-      <c r="H20" s="73"/>
+      <c r="D20" s="70"/>
+      <c r="E20" s="70"/>
+      <c r="F20" s="70"/>
+      <c r="G20" s="70"/>
+      <c r="H20" s="71"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="16" t="s">
@@ -4982,14 +4982,14 @@
       <c r="B21" s="17">
         <v>3</v>
       </c>
-      <c r="C21" s="71" t="s">
+      <c r="C21" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="72"/>
-      <c r="E21" s="72"/>
-      <c r="F21" s="72"/>
-      <c r="G21" s="72"/>
-      <c r="H21" s="73"/>
+      <c r="D21" s="70"/>
+      <c r="E21" s="70"/>
+      <c r="F21" s="70"/>
+      <c r="G21" s="70"/>
+      <c r="H21" s="71"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="16" t="s">
@@ -4998,14 +4998,14 @@
       <c r="B22" s="17">
         <v>1</v>
       </c>
-      <c r="C22" s="75" t="s">
+      <c r="C22" s="73" t="s">
         <v>32</v>
       </c>
-      <c r="D22" s="72"/>
-      <c r="E22" s="72"/>
-      <c r="F22" s="72"/>
-      <c r="G22" s="72"/>
-      <c r="H22" s="73"/>
+      <c r="D22" s="70"/>
+      <c r="E22" s="70"/>
+      <c r="F22" s="70"/>
+      <c r="G22" s="70"/>
+      <c r="H22" s="71"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="16" t="s">
@@ -5014,14 +5014,14 @@
       <c r="B23" s="17">
         <v>1</v>
       </c>
-      <c r="C23" s="71" t="s">
+      <c r="C23" s="69" t="s">
         <v>34</v>
       </c>
-      <c r="D23" s="72"/>
-      <c r="E23" s="72"/>
-      <c r="F23" s="72"/>
-      <c r="G23" s="72"/>
-      <c r="H23" s="73"/>
+      <c r="D23" s="70"/>
+      <c r="E23" s="70"/>
+      <c r="F23" s="70"/>
+      <c r="G23" s="70"/>
+      <c r="H23" s="71"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="18" t="s">
@@ -5030,14 +5030,14 @@
       <c r="B24" s="19">
         <v>1</v>
       </c>
-      <c r="C24" s="75" t="s">
+      <c r="C24" s="73" t="s">
         <v>36</v>
       </c>
-      <c r="D24" s="72"/>
-      <c r="E24" s="72"/>
-      <c r="F24" s="72"/>
-      <c r="G24" s="72"/>
-      <c r="H24" s="73"/>
+      <c r="D24" s="70"/>
+      <c r="E24" s="70"/>
+      <c r="F24" s="70"/>
+      <c r="G24" s="70"/>
+      <c r="H24" s="71"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="20" t="s">
@@ -5046,26 +5046,26 @@
       <c r="B25" s="21">
         <v>1</v>
       </c>
-      <c r="C25" s="71" t="s">
+      <c r="C25" s="69" t="s">
         <v>38</v>
       </c>
-      <c r="D25" s="72"/>
-      <c r="E25" s="72"/>
-      <c r="F25" s="72"/>
-      <c r="G25" s="72"/>
-      <c r="H25" s="73"/>
+      <c r="D25" s="70"/>
+      <c r="E25" s="70"/>
+      <c r="F25" s="70"/>
+      <c r="G25" s="70"/>
+      <c r="H25" s="71"/>
     </row>
     <row r="28" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="69" t="s">
+      <c r="A28" s="74" t="s">
         <v>39</v>
       </c>
-      <c r="B28" s="70"/>
-      <c r="C28" s="70"/>
-      <c r="D28" s="70"/>
-      <c r="E28" s="70"/>
-      <c r="F28" s="70"/>
-      <c r="G28" s="70"/>
-      <c r="H28" s="70"/>
+      <c r="B28" s="72"/>
+      <c r="C28" s="72"/>
+      <c r="D28" s="72"/>
+      <c r="E28" s="72"/>
+      <c r="F28" s="72"/>
+      <c r="G28" s="72"/>
+      <c r="H28" s="72"/>
     </row>
     <row r="29" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -5209,12 +5209,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="C10:H10"/>
-    <mergeCell ref="C21:H21"/>
-    <mergeCell ref="C9:H9"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="C23:H23"/>
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="C19:H19"/>
     <mergeCell ref="A1:H1"/>
@@ -5231,6 +5225,12 @@
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="C6:H6"/>
     <mergeCell ref="C24:H24"/>
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="C21:H21"/>
+    <mergeCell ref="C9:H9"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C23:H23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10979,141 +10979,141 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="83" t="s">
+      <c r="A1" s="80" t="s">
         <v>400</v>
       </c>
-      <c r="B1" s="70"/>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="69" t="s">
+      <c r="A3" s="74" t="s">
         <v>401</v>
       </c>
-      <c r="B3" s="70"/>
-      <c r="C3" s="70"/>
-      <c r="D3" s="70"/>
-      <c r="E3" s="70"/>
+      <c r="B3" s="72"/>
+      <c r="C3" s="72"/>
+      <c r="D3" s="72"/>
+      <c r="E3" s="72"/>
     </row>
     <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="89" t="s">
+      <c r="A4" s="86" t="s">
         <v>402</v>
       </c>
-      <c r="B4" s="73"/>
-      <c r="C4" s="78" t="s">
+      <c r="B4" s="71"/>
+      <c r="C4" s="79" t="s">
         <v>403</v>
       </c>
-      <c r="D4" s="70"/>
-      <c r="E4" s="70"/>
+      <c r="D4" s="72"/>
+      <c r="E4" s="72"/>
     </row>
     <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="86" t="s">
+      <c r="A5" s="83" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="73"/>
-      <c r="C5" s="78" t="s">
+      <c r="B5" s="71"/>
+      <c r="C5" s="79" t="s">
         <v>404</v>
       </c>
-      <c r="D5" s="70"/>
-      <c r="E5" s="70"/>
+      <c r="D5" s="72"/>
+      <c r="E5" s="72"/>
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="84" t="s">
+      <c r="A6" s="81" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="73"/>
-      <c r="C6" s="78" t="s">
+      <c r="B6" s="71"/>
+      <c r="C6" s="79" t="s">
         <v>405</v>
       </c>
-      <c r="D6" s="70"/>
-      <c r="E6" s="70"/>
+      <c r="D6" s="72"/>
+      <c r="E6" s="72"/>
     </row>
     <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="85" t="s">
+      <c r="A7" s="82" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="73"/>
-      <c r="C7" s="78" t="s">
+      <c r="B7" s="71"/>
+      <c r="C7" s="79" t="s">
         <v>406</v>
       </c>
-      <c r="D7" s="70"/>
-      <c r="E7" s="70"/>
+      <c r="D7" s="72"/>
+      <c r="E7" s="72"/>
     </row>
     <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="88" t="s">
+      <c r="A8" s="85" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="73"/>
-      <c r="C8" s="78" t="s">
+      <c r="B8" s="71"/>
+      <c r="C8" s="79" t="s">
         <v>407</v>
       </c>
-      <c r="D8" s="70"/>
-      <c r="E8" s="70"/>
+      <c r="D8" s="72"/>
+      <c r="E8" s="72"/>
     </row>
     <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="81" t="s">
+      <c r="A9" s="89" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="73"/>
-      <c r="C9" s="78" t="s">
+      <c r="B9" s="71"/>
+      <c r="C9" s="79" t="s">
         <v>408</v>
       </c>
-      <c r="D9" s="70"/>
-      <c r="E9" s="70"/>
+      <c r="D9" s="72"/>
+      <c r="E9" s="72"/>
     </row>
     <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="79" t="s">
+      <c r="A10" s="87" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="73"/>
-      <c r="C10" s="78" t="s">
+      <c r="B10" s="71"/>
+      <c r="C10" s="79" t="s">
         <v>409</v>
       </c>
-      <c r="D10" s="70"/>
-      <c r="E10" s="70"/>
+      <c r="D10" s="72"/>
+      <c r="E10" s="72"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="69" t="s">
+      <c r="A12" s="74" t="s">
         <v>410</v>
       </c>
-      <c r="B12" s="70"/>
-      <c r="C12" s="70"/>
-      <c r="D12" s="70"/>
-      <c r="E12" s="70"/>
+      <c r="B12" s="72"/>
+      <c r="C12" s="72"/>
+      <c r="D12" s="72"/>
+      <c r="E12" s="72"/>
     </row>
     <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="80" t="s">
+      <c r="A13" s="88" t="s">
         <v>411</v>
       </c>
-      <c r="B13" s="73"/>
-      <c r="C13" s="78" t="s">
+      <c r="B13" s="71"/>
+      <c r="C13" s="79" t="s">
         <v>412</v>
       </c>
-      <c r="D13" s="70"/>
-      <c r="E13" s="70"/>
+      <c r="D13" s="72"/>
+      <c r="E13" s="72"/>
     </row>
     <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="87" t="s">
+      <c r="A14" s="84" t="s">
         <v>413</v>
       </c>
-      <c r="B14" s="73"/>
-      <c r="C14" s="78" t="s">
+      <c r="B14" s="71"/>
+      <c r="C14" s="79" t="s">
         <v>414</v>
       </c>
-      <c r="D14" s="70"/>
-      <c r="E14" s="70"/>
+      <c r="D14" s="72"/>
+      <c r="E14" s="72"/>
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="82" t="s">
+      <c r="A15" s="78" t="s">
         <v>415</v>
       </c>
-      <c r="B15" s="73"/>
-      <c r="C15" s="78" t="s">
+      <c r="B15" s="71"/>
+      <c r="C15" s="79" t="s">
         <v>416</v>
       </c>
-      <c r="D15" s="70"/>
-      <c r="E15" s="70"/>
+      <c r="D15" s="72"/>
+      <c r="E15" s="72"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="47" t="s">
@@ -11128,6 +11128,13 @@
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C10:E10"/>
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="A1:E1"/>
@@ -11144,13 +11151,6 @@
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="C6:E6"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C10:E10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -11158,6 +11158,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ba695df1-2cef-45b3-b38e-525c8136ab22" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100052CBA820BEBCD468114CF62615C95D9" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="41d93ad2b4fecab14cfdaed9255371f8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ba695df1-2cef-45b3-b38e-525c8136ab22" xmlns:ns3="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="59a815193907c452009623866744c535" ns2:_="" ns3:_="">
     <xsd:import namespace="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
@@ -11398,27 +11418,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51CBE187-A7DE-4A9A-99BE-7485C92477B0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ba695df1-2cef-45b3-b38e-525c8136ab22" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A39E8DA8-D782-4F69-B46B-77021BF1B166}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82507086-9DCD-4197-A4F6-ECCED658E0D9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11435,29 +11460,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A39E8DA8-D782-4F69-B46B-77021BF1B166}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51CBE187-A7DE-4A9A-99BE-7485C92477B0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="ba695df1-2cef-45b3-b38e-525c8136ab22"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="d75fa1b2-e4ff-4c4f-9d1f-2231fcc7043e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>